<commit_message>
auto: actualizar BD BONOS CER.xlsx [2026-09-30]
</commit_message>
<xml_diff>
--- a/backend/data/BD BONOS CER.xlsx
+++ b/backend/data/BD BONOS CER.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -472,7 +472,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>X30S6</t>
+          <t>X30N6</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -482,16 +482,16 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>715.715236</v>
+        <v>659.678896</v>
       </c>
       <c r="F2" t="n">
         <v>100</v>
@@ -514,26 +514,26 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>X30N6</t>
+          <t>TZXO6</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>LECER</t>
+          <t>BONCER_ZC</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-11-30</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2025-11-28</t>
+          <t>2024-10-17</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>659.678896</v>
+        <v>480.152578</v>
       </c>
       <c r="F3" t="n">
         <v>100</v>
@@ -556,7 +556,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TZXO6</t>
+          <t>TZXD6</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -566,16 +566,16 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-12-15</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2024-10-17</t>
+          <t>2024-03-01</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>480.152578</v>
+        <v>271.047556</v>
       </c>
       <c r="F4" t="n">
         <v>100</v>
@@ -598,7 +598,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TZXD6</t>
+          <t>TZXM7</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -608,16 +608,16 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-12-15</t>
+          <t>2027-03-31</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2024-03-01</t>
+          <t>2024-05-06</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>271.047556</v>
+        <v>361.317603</v>
       </c>
       <c r="F5" t="n">
         <v>100</v>
@@ -640,7 +640,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>TZXM7</t>
+          <t>TZXA7</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -650,16 +650,16 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2027-03-31</t>
+          <t>2027-04-30</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2024-05-06</t>
+          <t>2025-11-12</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>361.317603</v>
+        <v>651.898062</v>
       </c>
       <c r="F6" t="n">
         <v>100</v>
@@ -682,7 +682,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TZXA7</t>
+          <t>TZXY7</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -692,7 +692,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2027-04-30</t>
+          <t>2027-05-31</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -724,7 +724,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>TZXY7</t>
+          <t>TZX27</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -734,16 +734,16 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2027-05-31</t>
+          <t>2027-06-30</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2025-11-12</t>
+          <t>2024-01-18</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>651.898062</v>
+        <v>200.388015</v>
       </c>
       <c r="F8" t="n">
         <v>100</v>
@@ -766,7 +766,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>TZX27</t>
+          <t>TZXS7</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -776,16 +776,16 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2027-06-30</t>
+          <t>2027-09-30</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2024-01-18</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>200.388015</v>
+        <v>715.715236</v>
       </c>
       <c r="F9" t="n">
         <v>100</v>
@@ -808,7 +808,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TZXS7</t>
+          <t>TZXD7</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -818,16 +818,16 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2027-09-30</t>
+          <t>2027-12-15</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2024-03-01</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>715.715236</v>
+        <v>271.047556</v>
       </c>
       <c r="F10" t="n">
         <v>100</v>
@@ -850,7 +850,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TZXD7</t>
+          <t>TZX28</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -860,16 +860,16 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2027-12-15</t>
+          <t>2028-06-30</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2024-03-01</t>
+          <t>2024-01-18</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>271.047556</v>
+        <v>200.388015</v>
       </c>
       <c r="F11" t="n">
         <v>100</v>
@@ -892,7 +892,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TZX28</t>
+          <t>TZXS8</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -902,16 +902,16 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2028-06-30</t>
+          <t>2028-09-29</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2024-01-18</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>200.388015</v>
+        <v>721.585027</v>
       </c>
       <c r="F12" t="n">
         <v>100</v>
@@ -934,7 +934,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TZXS8</t>
+          <t>TZXM9</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -944,7 +944,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2028-09-29</t>
+          <t>2029-03-28</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -976,26 +976,26 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>TZXM9</t>
+          <t>TX26</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>BONCER_ZC</t>
+          <t>BONCER_COUPON</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2029-03-28</t>
+          <t>2026-11-09</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2023-07-18</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>721.585027</v>
+        <v>113.059645</v>
       </c>
       <c r="F14" t="n">
         <v>100</v>
@@ -1004,10 +1004,10 @@
         <v>100</v>
       </c>
       <c r="H14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
@@ -1018,7 +1018,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>TX26</t>
+          <t>TX28</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1028,16 +1028,16 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-11-09</t>
+          <t>2028-11-09</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2023-07-18</t>
+          <t>2021-12-02</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>113.059645</v>
+        <v>37.587966</v>
       </c>
       <c r="F15" t="n">
         <v>100</v>
@@ -1046,7 +1046,7 @@
         <v>100</v>
       </c>
       <c r="H15" t="n">
-        <v>2</v>
+        <v>2.25</v>
       </c>
       <c r="I15" t="n">
         <v>2</v>
@@ -1060,7 +1060,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>TX28</t>
+          <t>TX31</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1070,16 +1070,16 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2028-11-09</t>
+          <t>2031-11-30</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2021-12-02</t>
+          <t>2022-05-11</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>37.587966</v>
+        <v>46.710616</v>
       </c>
       <c r="F16" t="n">
         <v>100</v>
@@ -1088,7 +1088,7 @@
         <v>100</v>
       </c>
       <c r="H16" t="n">
-        <v>2.25</v>
+        <v>2.5</v>
       </c>
       <c r="I16" t="n">
         <v>2</v>
@@ -1102,26 +1102,26 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>TX31</t>
+          <t>TZXM8</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>BONCER_COUPON</t>
+          <t>BONCER_ZC</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2031-11-30</t>
+          <t>2028-03-31</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2022-05-11</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>46.710616</v>
+        <v>721.585027</v>
       </c>
       <c r="F17" t="n">
         <v>100</v>
@@ -1130,10 +1130,10 @@
         <v>100</v>
       </c>
       <c r="H17" t="n">
-        <v>2.5</v>
+        <v>0</v>
       </c>
       <c r="I17" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
@@ -1144,7 +1144,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>TZXM8</t>
+          <t>TXM8</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1154,16 +1154,16 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2028-03-31</t>
+          <t>2028-06-30</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>721.585027</v>
+        <v>761.505166</v>
       </c>
       <c r="F18" t="n">
         <v>100</v>
@@ -1186,7 +1186,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>TXM8</t>
+          <t>TXM9</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1196,16 +1196,16 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2028-06-30</t>
+          <t>2029-06-29</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>761.505166</v>
+        <v>746.3809230000001</v>
       </c>
       <c r="F19" t="n">
         <v>100</v>
@@ -1220,48 +1220,6 @@
         <v>0</v>
       </c>
       <c r="J19" t="inlineStr">
-        <is>
-          <t>business_days_before:10</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>TXM9</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>BONCER_ZC</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>2029-06-29</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>2026-04-16</t>
-        </is>
-      </c>
-      <c r="E20" t="n">
-        <v>746.3809230000001</v>
-      </c>
-      <c r="F20" t="n">
-        <v>100</v>
-      </c>
-      <c r="G20" t="n">
-        <v>100</v>
-      </c>
-      <c r="H20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I20" t="n">
-        <v>0</v>
-      </c>
-      <c r="J20" t="inlineStr">
         <is>
           <t>business_days_before:10</t>
         </is>
@@ -1278,7 +1236,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C58"/>
+  <dimension ref="A1:C57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1301,12 +1259,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>X30S6</t>
+          <t>X30N6</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -1316,12 +1274,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>X30N6</t>
+          <t>TZXO6</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-11-30</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -1331,12 +1289,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TZXO6</t>
+          <t>TZXD6</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-12-15</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1346,12 +1304,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TZXD6</t>
+          <t>TZXM7</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-12-15</t>
+          <t>2027-03-31</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1361,12 +1319,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>TZXM7</t>
+          <t>TZXA7</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2027-03-31</t>
+          <t>2027-04-30</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1376,12 +1334,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TZXA7</t>
+          <t>TZXY7</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2027-04-30</t>
+          <t>2027-05-31</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1391,12 +1349,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>TZXY7</t>
+          <t>TZX27</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2027-05-31</t>
+          <t>2027-06-30</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1406,12 +1364,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>TZX27</t>
+          <t>TZXS7</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2027-06-30</t>
+          <t>2027-09-30</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1421,12 +1379,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TZXS7</t>
+          <t>TZXD7</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2027-09-30</t>
+          <t>2027-12-15</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1436,12 +1394,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TZXD7</t>
+          <t>TZX28</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2027-12-15</t>
+          <t>2028-06-30</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1451,12 +1409,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TZX28</t>
+          <t>TZXS8</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2028-06-30</t>
+          <t>2028-09-29</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1466,12 +1424,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TZXS8</t>
+          <t>TZXM9</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2028-09-29</t>
+          <t>2029-03-28</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -1481,16 +1439,16 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>TZXM9</t>
+          <t>TX26</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2029-03-28</t>
+          <t>2023-11-09</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -1501,7 +1459,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2023-11-09</t>
+          <t>2024-05-09</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -1516,7 +1474,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2024-05-09</t>
+          <t>2024-11-09</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -1531,7 +1489,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2024-11-09</t>
+          <t>2025-05-09</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -1546,7 +1504,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2025-05-09</t>
+          <t>2025-11-09</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -1561,7 +1519,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2025-11-09</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -1576,26 +1534,26 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-11-09</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>1</v>
+        <v>101</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>TX26</t>
+          <t>TX28</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-11-09</t>
+          <t>2022-05-09</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>101</v>
+        <v>1.125</v>
       </c>
     </row>
     <row r="22">
@@ -1606,7 +1564,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2022-05-09</t>
+          <t>2022-11-09</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -1621,7 +1579,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2022-11-09</t>
+          <t>2023-05-09</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -1636,7 +1594,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2023-05-09</t>
+          <t>2023-11-09</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -1651,7 +1609,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2023-11-09</t>
+          <t>2024-05-09</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -1666,7 +1624,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2024-05-09</t>
+          <t>2024-11-09</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -1681,7 +1639,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2024-11-09</t>
+          <t>2025-05-09</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -1696,7 +1654,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2025-05-09</t>
+          <t>2025-11-09</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -1711,7 +1669,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2025-11-09</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -1726,7 +1684,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-11-09</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -1741,7 +1699,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-11-09</t>
+          <t>2027-05-09</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -1756,7 +1714,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2027-05-09</t>
+          <t>2027-11-09</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -1771,7 +1729,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2027-11-09</t>
+          <t>2028-05-09</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -1786,26 +1744,26 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2028-05-09</t>
+          <t>2028-11-09</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>1.125</v>
+        <v>101.125</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>TX28</t>
+          <t>TX31</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2028-11-09</t>
+          <t>2022-05-30</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>101.125</v>
+        <v>1.25</v>
       </c>
     </row>
     <row r="36">
@@ -1816,7 +1774,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2022-05-30</t>
+          <t>2022-11-30</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -1831,7 +1789,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2022-11-30</t>
+          <t>2023-05-30</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -1846,7 +1804,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2023-05-30</t>
+          <t>2023-11-30</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -1861,7 +1819,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2023-11-30</t>
+          <t>2024-05-30</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -1876,7 +1834,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2024-05-30</t>
+          <t>2024-11-30</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -1891,7 +1849,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2024-11-30</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -1906,7 +1864,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2025-05-30</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -1921,7 +1879,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2025-11-30</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -1936,7 +1894,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -1951,7 +1909,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-11-30</t>
+          <t>2027-05-30</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -1966,7 +1924,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2027-05-30</t>
+          <t>2027-11-30</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -1981,7 +1939,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2027-11-30</t>
+          <t>2028-05-30</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -1996,7 +1954,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2028-05-30</t>
+          <t>2028-11-30</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -2011,7 +1969,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2028-11-30</t>
+          <t>2029-05-30</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -2026,7 +1984,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2029-05-30</t>
+          <t>2029-11-30</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -2041,7 +1999,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2029-11-30</t>
+          <t>2030-05-30</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -2056,7 +2014,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2030-05-30</t>
+          <t>2030-11-30</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -2071,7 +2029,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2030-11-30</t>
+          <t>2031-05-30</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -2086,37 +2044,37 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2031-05-30</t>
+          <t>2031-11-30</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>1.25</v>
+        <v>101.25</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>TX31</t>
+          <t>TZXM8</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2031-11-30</t>
+          <t>2028-03-31</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>101.25</v>
+        <v>100</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>TZXM8</t>
+          <t>TXM8</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2028-03-31</t>
+          <t>2028-06-30</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -2126,30 +2084,15 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>TXM8</t>
+          <t>TXM9</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2028-06-30</t>
+          <t>2029-06-29</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>TXM9</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>2029-06-29</t>
-        </is>
-      </c>
-      <c r="C58" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: actualizar BD BONOS CER.xlsx [2026-10-30]
</commit_message>
<xml_diff>
--- a/backend/data/BD BONOS CER.xlsx
+++ b/backend/data/BD BONOS CER.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -514,7 +514,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TZXO6</t>
+          <t>TZXD6</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -524,16 +524,16 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-12-15</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2024-10-17</t>
+          <t>2024-03-01</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>480.152578</v>
+        <v>271.047556</v>
       </c>
       <c r="F3" t="n">
         <v>100</v>
@@ -556,7 +556,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TZXD6</t>
+          <t>TZXM7</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -566,16 +566,16 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-12-15</t>
+          <t>2027-03-31</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2024-03-01</t>
+          <t>2024-05-06</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>271.047556</v>
+        <v>361.317603</v>
       </c>
       <c r="F4" t="n">
         <v>100</v>
@@ -598,7 +598,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TZXM7</t>
+          <t>TZXA7</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -608,16 +608,16 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2027-03-31</t>
+          <t>2027-04-30</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2024-05-06</t>
+          <t>2025-11-12</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>361.317603</v>
+        <v>651.898062</v>
       </c>
       <c r="F5" t="n">
         <v>100</v>
@@ -640,7 +640,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>TZXA7</t>
+          <t>TZXY7</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -650,7 +650,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2027-04-30</t>
+          <t>2027-05-31</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TZXY7</t>
+          <t>TZX27</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -692,16 +692,16 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2027-05-31</t>
+          <t>2027-06-30</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2025-11-12</t>
+          <t>2024-01-18</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>651.898062</v>
+        <v>200.388015</v>
       </c>
       <c r="F7" t="n">
         <v>100</v>
@@ -724,7 +724,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>TZX27</t>
+          <t>TZXS7</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -734,16 +734,16 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2027-06-30</t>
+          <t>2027-09-30</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2024-01-18</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>200.388015</v>
+        <v>715.715236</v>
       </c>
       <c r="F8" t="n">
         <v>100</v>
@@ -766,7 +766,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>TZXS7</t>
+          <t>TZXD7</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -776,16 +776,16 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2027-09-30</t>
+          <t>2027-12-15</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2024-03-01</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>715.715236</v>
+        <v>271.047556</v>
       </c>
       <c r="F9" t="n">
         <v>100</v>
@@ -808,7 +808,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TZXD7</t>
+          <t>TZX28</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -818,16 +818,16 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2027-12-15</t>
+          <t>2028-06-30</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2024-03-01</t>
+          <t>2024-01-18</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>271.047556</v>
+        <v>200.388015</v>
       </c>
       <c r="F10" t="n">
         <v>100</v>
@@ -850,7 +850,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TZX28</t>
+          <t>TZXS8</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -860,16 +860,16 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2028-06-30</t>
+          <t>2028-09-29</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2024-01-18</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>200.388015</v>
+        <v>721.585027</v>
       </c>
       <c r="F11" t="n">
         <v>100</v>
@@ -892,7 +892,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TZXS8</t>
+          <t>TZXM9</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -902,7 +902,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2028-09-29</t>
+          <t>2029-03-28</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -934,26 +934,26 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TZXM9</t>
+          <t>TX26</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>BONCER_ZC</t>
+          <t>BONCER_COUPON</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2029-03-28</t>
+          <t>2026-11-09</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2023-07-18</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>721.585027</v>
+        <v>113.059645</v>
       </c>
       <c r="F13" t="n">
         <v>100</v>
@@ -962,10 +962,10 @@
         <v>100</v>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
@@ -976,7 +976,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>TX26</t>
+          <t>TX28</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -986,16 +986,16 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-11-09</t>
+          <t>2028-11-09</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2023-07-18</t>
+          <t>2021-12-02</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>113.059645</v>
+        <v>37.587966</v>
       </c>
       <c r="F14" t="n">
         <v>100</v>
@@ -1004,7 +1004,7 @@
         <v>100</v>
       </c>
       <c r="H14" t="n">
-        <v>2</v>
+        <v>2.25</v>
       </c>
       <c r="I14" t="n">
         <v>2</v>
@@ -1018,7 +1018,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>TX28</t>
+          <t>TX31</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1028,16 +1028,16 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2028-11-09</t>
+          <t>2031-11-30</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2021-12-02</t>
+          <t>2022-05-11</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>37.587966</v>
+        <v>46.710616</v>
       </c>
       <c r="F15" t="n">
         <v>100</v>
@@ -1046,7 +1046,7 @@
         <v>100</v>
       </c>
       <c r="H15" t="n">
-        <v>2.25</v>
+        <v>2.5</v>
       </c>
       <c r="I15" t="n">
         <v>2</v>
@@ -1060,26 +1060,26 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>TX31</t>
+          <t>TZXM8</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>BONCER_COUPON</t>
+          <t>BONCER_ZC</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2031-11-30</t>
+          <t>2028-03-31</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2022-05-11</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>46.710616</v>
+        <v>721.585027</v>
       </c>
       <c r="F16" t="n">
         <v>100</v>
@@ -1088,10 +1088,10 @@
         <v>100</v>
       </c>
       <c r="H16" t="n">
-        <v>2.5</v>
+        <v>0</v>
       </c>
       <c r="I16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
@@ -1102,7 +1102,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>TZXM8</t>
+          <t>TXM8</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1112,16 +1112,16 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2028-03-31</t>
+          <t>2028-06-30</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>721.585027</v>
+        <v>761.505166</v>
       </c>
       <c r="F17" t="n">
         <v>100</v>
@@ -1144,7 +1144,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>TXM8</t>
+          <t>TXM9</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1154,16 +1154,16 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2028-06-30</t>
+          <t>2029-06-29</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>761.505166</v>
+        <v>746.3809230000001</v>
       </c>
       <c r="F18" t="n">
         <v>100</v>
@@ -1178,48 +1178,6 @@
         <v>0</v>
       </c>
       <c r="J18" t="inlineStr">
-        <is>
-          <t>business_days_before:10</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>TXM9</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>BONCER_ZC</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>2029-06-29</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>2026-04-16</t>
-        </is>
-      </c>
-      <c r="E19" t="n">
-        <v>746.3809230000001</v>
-      </c>
-      <c r="F19" t="n">
-        <v>100</v>
-      </c>
-      <c r="G19" t="n">
-        <v>100</v>
-      </c>
-      <c r="H19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" t="inlineStr">
         <is>
           <t>business_days_before:10</t>
         </is>
@@ -1236,7 +1194,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C57"/>
+  <dimension ref="A1:C56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1274,12 +1232,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TZXO6</t>
+          <t>TZXD6</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-12-15</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -1289,12 +1247,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TZXD6</t>
+          <t>TZXM7</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-12-15</t>
+          <t>2027-03-31</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1304,12 +1262,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TZXM7</t>
+          <t>TZXA7</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2027-03-31</t>
+          <t>2027-04-30</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1319,12 +1277,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>TZXA7</t>
+          <t>TZXY7</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2027-04-30</t>
+          <t>2027-05-31</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1334,12 +1292,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TZXY7</t>
+          <t>TZX27</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2027-05-31</t>
+          <t>2027-06-30</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1349,12 +1307,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>TZX27</t>
+          <t>TZXS7</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2027-06-30</t>
+          <t>2027-09-30</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1364,12 +1322,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>TZXS7</t>
+          <t>TZXD7</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2027-09-30</t>
+          <t>2027-12-15</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1379,12 +1337,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TZXD7</t>
+          <t>TZX28</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2027-12-15</t>
+          <t>2028-06-30</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1394,12 +1352,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TZX28</t>
+          <t>TZXS8</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2028-06-30</t>
+          <t>2028-09-29</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1409,12 +1367,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TZXS8</t>
+          <t>TZXM9</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2028-09-29</t>
+          <t>2029-03-28</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1424,16 +1382,16 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TZXM9</t>
+          <t>TX26</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2029-03-28</t>
+          <t>2023-11-09</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -1444,7 +1402,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2023-11-09</t>
+          <t>2024-05-09</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -1459,7 +1417,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2024-05-09</t>
+          <t>2024-11-09</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -1474,7 +1432,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2024-11-09</t>
+          <t>2025-05-09</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -1489,7 +1447,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2025-05-09</t>
+          <t>2025-11-09</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -1504,7 +1462,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2025-11-09</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -1519,26 +1477,26 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-11-09</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>1</v>
+        <v>101</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TX26</t>
+          <t>TX28</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-11-09</t>
+          <t>2022-05-09</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>101</v>
+        <v>1.125</v>
       </c>
     </row>
     <row r="21">
@@ -1549,7 +1507,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2022-05-09</t>
+          <t>2022-11-09</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -1564,7 +1522,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2022-11-09</t>
+          <t>2023-05-09</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -1579,7 +1537,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2023-05-09</t>
+          <t>2023-11-09</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -1594,7 +1552,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2023-11-09</t>
+          <t>2024-05-09</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -1609,7 +1567,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2024-05-09</t>
+          <t>2024-11-09</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -1624,7 +1582,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2024-11-09</t>
+          <t>2025-05-09</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -1639,7 +1597,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2025-05-09</t>
+          <t>2025-11-09</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -1654,7 +1612,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2025-11-09</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -1669,7 +1627,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-11-09</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -1684,7 +1642,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-11-09</t>
+          <t>2027-05-09</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -1699,7 +1657,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2027-05-09</t>
+          <t>2027-11-09</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -1714,7 +1672,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2027-11-09</t>
+          <t>2028-05-09</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -1729,26 +1687,26 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2028-05-09</t>
+          <t>2028-11-09</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>1.125</v>
+        <v>101.125</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>TX28</t>
+          <t>TX31</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2028-11-09</t>
+          <t>2022-05-30</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>101.125</v>
+        <v>1.25</v>
       </c>
     </row>
     <row r="35">
@@ -1759,7 +1717,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2022-05-30</t>
+          <t>2022-11-30</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -1774,7 +1732,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2022-11-30</t>
+          <t>2023-05-30</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -1789,7 +1747,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2023-05-30</t>
+          <t>2023-11-30</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -1804,7 +1762,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2023-11-30</t>
+          <t>2024-05-30</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -1819,7 +1777,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2024-05-30</t>
+          <t>2024-11-30</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -1834,7 +1792,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2024-11-30</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -1849,7 +1807,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2025-05-30</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -1864,7 +1822,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2025-11-30</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -1879,7 +1837,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -1894,7 +1852,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-11-30</t>
+          <t>2027-05-30</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -1909,7 +1867,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2027-05-30</t>
+          <t>2027-11-30</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -1924,7 +1882,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2027-11-30</t>
+          <t>2028-05-30</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -1939,7 +1897,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2028-05-30</t>
+          <t>2028-11-30</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -1954,7 +1912,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2028-11-30</t>
+          <t>2029-05-30</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -1969,7 +1927,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2029-05-30</t>
+          <t>2029-11-30</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -1984,7 +1942,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2029-11-30</t>
+          <t>2030-05-30</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -1999,7 +1957,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2030-05-30</t>
+          <t>2030-11-30</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -2014,7 +1972,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2030-11-30</t>
+          <t>2031-05-30</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -2029,37 +1987,37 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2031-05-30</t>
+          <t>2031-11-30</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>1.25</v>
+        <v>101.25</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>TX31</t>
+          <t>TZXM8</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2031-11-30</t>
+          <t>2028-03-31</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>101.25</v>
+        <v>100</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>TZXM8</t>
+          <t>TXM8</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2028-03-31</t>
+          <t>2028-06-30</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -2069,30 +2027,15 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>TXM8</t>
+          <t>TXM9</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2028-06-30</t>
+          <t>2029-06-29</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>TXM9</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>2029-06-29</t>
-        </is>
-      </c>
-      <c r="C57" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>